<commit_message>
server created using http
</commit_message>
<xml_diff>
--- a/topics covered.xlsx
+++ b/topics covered.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t xml:space="preserve">basics </t>
   </si>
@@ -39,6 +39,18 @@
   </si>
   <si>
     <t>require()</t>
+  </si>
+  <si>
+    <t>importing</t>
+  </si>
+  <si>
+    <t>exporting modules</t>
+  </si>
+  <si>
+    <t>fs.readFileSync()</t>
+  </si>
+  <si>
+    <t>fs.writeFileSync()</t>
   </si>
 </sst>
 </file>
@@ -368,6 +380,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="3:5" x14ac:dyDescent="0.35">
@@ -375,30 +388,40 @@
         <v>46199</v>
       </c>
       <c r="D5" s="1">
-        <v>46200</v>
-      </c>
-      <c r="E5" s="1">
-        <v>46201</v>
-      </c>
+        <v>46206</v>
+      </c>
+      <c r="E5" s="1"/>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>0</v>
       </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
         <v>1</v>
       </c>
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
         <v>4</v>
       </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
         <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.35">

</xml_diff>